<commit_message>
updated datasets and figures for Ecosphere R1
</commit_message>
<xml_diff>
--- a/data/2022-03-03_LakeErie_Mastersheet.xlsx
+++ b/data/2022-03-03_LakeErie_Mastersheet.xlsx
@@ -1,29 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://trentu-my.sharepoint.com/personal/sandraklemet_trentu_ca/Documents/Documents/Etudes/Trent/Xenopoulos lab/Projects/LakeErie_animal-excretion/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="488" documentId="13_ncr:1_{EA2E9A16-F367-47E5-9F32-F761EF32E94C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{552A0181-A305-432F-B9D4-93FBCBBED485}"/>
+  <xr:revisionPtr revIDLastSave="811" documentId="13_ncr:1_{EA2E9A16-F367-47E5-9F32-F761EF32E94C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4FF3B61A-11A6-49B6-B083-1D9F36069336}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="6" xr2:uid="{FCD5901F-55C5-46A6-83E9-A175C073FB2F}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="3" activeTab="3" xr2:uid="{FCD5901F-55C5-46A6-83E9-A175C073FB2F}"/>
   </bookViews>
   <sheets>
     <sheet name="Fishing and Environmental data" sheetId="3" r:id="rId1"/>
-    <sheet name="Fish and mussel sampling" sheetId="1" r:id="rId2"/>
-    <sheet name="Fish_biomass_estimates" sheetId="5" r:id="rId3"/>
-    <sheet name="Dreissenid_biomass_estimates" sheetId="6" r:id="rId4"/>
-    <sheet name="WesternBasin_biomass" sheetId="7" r:id="rId5"/>
-    <sheet name="Column headings" sheetId="4" r:id="rId6"/>
-    <sheet name="21 08 26 Lake Erie Mastersheet" sheetId="2" r:id="rId7"/>
+    <sheet name="Fish_species_biomass_estimates" sheetId="5" r:id="rId2"/>
+    <sheet name="Fish and mussel sampling" sheetId="1" r:id="rId3"/>
+    <sheet name="Dreissenid_biomass_visestimates" sheetId="6" r:id="rId4"/>
+    <sheet name="Dreissenid_biomass_digestimates" sheetId="8" r:id="rId5"/>
+    <sheet name="Fish_total_WB_biomass_LEBS" sheetId="9" r:id="rId6"/>
+    <sheet name="WesternBasin_total_biomass" sheetId="7" r:id="rId7"/>
+    <sheet name="Column headings" sheetId="4" r:id="rId8"/>
+    <sheet name="21 08 26 Lake Erie Mastersheet" sheetId="2" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'21 08 26 Lake Erie Mastersheet'!$A$1:$CJ$160</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Fish and mussel sampling'!$A$1:$L$160</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'21 08 26 Lake Erie Mastersheet'!$A$1:$CJ$160</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Fish and mussel sampling'!$A$1:$L$160</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -44,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2351" uniqueCount="223">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2390" uniqueCount="251">
   <si>
     <t>Sampling run</t>
   </si>
@@ -505,9 +507,6 @@
     <t>Year</t>
   </si>
   <si>
-    <t>Biomass (kg/ha)</t>
-  </si>
-  <si>
     <t>Cecilia, Aaron, Claire, James, Sandra</t>
   </si>
   <si>
@@ -703,23 +702,110 @@
     <t>Source</t>
   </si>
   <si>
+    <t>Biomass_lakewide (kg/ha)</t>
+  </si>
+  <si>
+    <t>Biomass_WB (kg/ha)</t>
+  </si>
+  <si>
+    <t>n</t>
+  </si>
+  <si>
+    <t>1992</t>
+  </si>
+  <si>
+    <t>1993</t>
+  </si>
+  <si>
+    <t>1998</t>
+  </si>
+  <si>
+    <t>2002</t>
+  </si>
+  <si>
+    <t>2011</t>
+  </si>
+  <si>
+    <t>2014</t>
+  </si>
+  <si>
+    <t>2019</t>
+  </si>
+  <si>
+    <t>2004</t>
+  </si>
+  <si>
+    <t>sqrt(((n1 - 1)*sd1^2 + (n2 - 1)*sd2^2) / (n1 + n2 - 2))</t>
+  </si>
+  <si>
+    <t>n_spring</t>
+  </si>
+  <si>
+    <t>n_autumn</t>
+  </si>
+  <si>
+    <t>Pooled SD calculation</t>
+  </si>
+  <si>
+    <t>biomass_spring_kg_ha</t>
+  </si>
+  <si>
+    <t>biomass_autumn_kg_ha</t>
+  </si>
+  <si>
+    <t>biomass_spring_kg_ha_se</t>
+  </si>
+  <si>
+    <t>biomass_autumn_kg_ha_se</t>
+  </si>
+  <si>
+    <t>biomass_spring_kg_ha_sd</t>
+  </si>
+  <si>
+    <t>biomass_autumn_kg_ha_sd</t>
+  </si>
+  <si>
+    <t>biomas_kg_ha_pooled_sd</t>
+  </si>
+  <si>
+    <t>biomass_mean_kg_ha</t>
+  </si>
+  <si>
+    <t>n.b.total</t>
+  </si>
+  <si>
+    <t>n.b.spring</t>
+  </si>
+  <si>
+    <t>n.b.autumn</t>
+  </si>
+  <si>
+    <t>biomass.kg.ha</t>
+  </si>
+  <si>
+    <t>biomass.g.m2</t>
+  </si>
+  <si>
+    <t>biomass.kg.ha.sd</t>
+  </si>
+  <si>
+    <t>biomass.g.m2.sd</t>
+  </si>
+  <si>
+    <t>biomass.g.m2.se</t>
+  </si>
+  <si>
     <t>Fish</t>
   </si>
   <si>
     <t>Dreissenid</t>
-  </si>
-  <si>
-    <t>Biomass (kg/ha) SD</t>
-  </si>
-  <si>
-    <t>Biomass (g/m2) SD</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -762,6 +848,27 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -784,7 +891,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -801,6 +908,18 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="11" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1151,7 +1270,7 @@
         <v>7</v>
       </c>
       <c r="J1" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="K1" t="s">
         <v>8</v>
@@ -1166,163 +1285,163 @@
         <v>36</v>
       </c>
       <c r="O1" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="P1" t="s">
+        <v>158</v>
+      </c>
+      <c r="Q1" t="s">
         <v>159</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>160</v>
       </c>
       <c r="R1" t="s">
         <v>97</v>
       </c>
       <c r="S1" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="T1" t="s">
+        <v>160</v>
+      </c>
+      <c r="U1" t="s">
         <v>161</v>
       </c>
-      <c r="U1" t="s">
+      <c r="V1" t="s">
         <v>162</v>
       </c>
-      <c r="V1" t="s">
+      <c r="W1" t="s">
         <v>163</v>
       </c>
-      <c r="W1" t="s">
+      <c r="X1" t="s">
         <v>164</v>
       </c>
-      <c r="X1" t="s">
+      <c r="Y1" t="s">
         <v>165</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Z1" t="s">
         <v>166</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="AA1" t="s">
         <v>167</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AB1" t="s">
         <v>168</v>
       </c>
-      <c r="AB1" t="s">
+      <c r="AC1" t="s">
         <v>169</v>
       </c>
-      <c r="AC1" t="s">
+      <c r="AD1" t="s">
         <v>170</v>
       </c>
-      <c r="AD1" t="s">
+      <c r="AE1" t="s">
         <v>171</v>
       </c>
-      <c r="AE1" t="s">
+      <c r="AF1" t="s">
         <v>172</v>
       </c>
-      <c r="AF1" t="s">
+      <c r="AG1" t="s">
         <v>173</v>
       </c>
-      <c r="AG1" t="s">
+      <c r="AH1" t="s">
         <v>174</v>
       </c>
-      <c r="AH1" t="s">
+      <c r="AI1" t="s">
         <v>175</v>
       </c>
-      <c r="AI1" t="s">
+      <c r="AJ1" t="s">
         <v>176</v>
       </c>
-      <c r="AJ1" t="s">
+      <c r="AK1" t="s">
         <v>177</v>
       </c>
-      <c r="AK1" t="s">
+      <c r="AL1" t="s">
         <v>178</v>
       </c>
-      <c r="AL1" t="s">
+      <c r="AM1" t="s">
         <v>179</v>
       </c>
-      <c r="AM1" t="s">
+      <c r="AN1" t="s">
         <v>180</v>
       </c>
-      <c r="AN1" t="s">
+      <c r="AO1" t="s">
         <v>181</v>
       </c>
-      <c r="AO1" t="s">
+      <c r="AP1" t="s">
         <v>182</v>
       </c>
-      <c r="AP1" t="s">
+      <c r="AQ1" t="s">
         <v>183</v>
       </c>
-      <c r="AQ1" t="s">
+      <c r="AR1" t="s">
         <v>184</v>
       </c>
-      <c r="AR1" t="s">
+      <c r="AS1" t="s">
         <v>185</v>
       </c>
-      <c r="AS1" t="s">
+      <c r="AT1" t="s">
         <v>186</v>
       </c>
-      <c r="AT1" t="s">
+      <c r="AU1" t="s">
         <v>187</v>
       </c>
-      <c r="AU1" t="s">
+      <c r="AV1" t="s">
         <v>188</v>
       </c>
-      <c r="AV1" t="s">
+      <c r="AW1" t="s">
         <v>189</v>
       </c>
-      <c r="AW1" t="s">
+      <c r="AX1" t="s">
         <v>190</v>
       </c>
-      <c r="AX1" t="s">
+      <c r="AY1" t="s">
         <v>191</v>
       </c>
-      <c r="AY1" t="s">
+      <c r="AZ1" t="s">
         <v>192</v>
       </c>
-      <c r="AZ1" t="s">
+      <c r="BA1" t="s">
         <v>193</v>
       </c>
-      <c r="BA1" t="s">
+      <c r="BB1" t="s">
         <v>194</v>
       </c>
-      <c r="BB1" t="s">
+      <c r="BC1" t="s">
         <v>195</v>
       </c>
-      <c r="BC1" t="s">
+      <c r="BD1" t="s">
         <v>196</v>
       </c>
-      <c r="BD1" t="s">
+      <c r="BE1" t="s">
         <v>197</v>
       </c>
-      <c r="BE1" t="s">
+      <c r="BF1" t="s">
         <v>198</v>
       </c>
-      <c r="BF1" t="s">
+      <c r="BG1" t="s">
         <v>199</v>
       </c>
-      <c r="BG1" t="s">
+      <c r="BH1" t="s">
         <v>200</v>
       </c>
-      <c r="BH1" t="s">
+      <c r="BI1" t="s">
         <v>201</v>
       </c>
-      <c r="BI1" t="s">
+      <c r="BJ1" t="s">
         <v>202</v>
       </c>
-      <c r="BJ1" t="s">
+      <c r="BK1" t="s">
         <v>203</v>
       </c>
-      <c r="BK1" t="s">
+      <c r="BL1" t="s">
         <v>204</v>
       </c>
-      <c r="BL1" t="s">
+      <c r="BM1" t="s">
         <v>205</v>
       </c>
-      <c r="BM1" t="s">
+      <c r="BN1" t="s">
         <v>206</v>
       </c>
-      <c r="BN1" t="s">
+      <c r="BO1" t="s">
         <v>207</v>
-      </c>
-      <c r="BO1" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="2" spans="1:67" x14ac:dyDescent="0.35">
@@ -1354,16 +1473,16 @@
         <v>43</v>
       </c>
       <c r="N2" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="O2">
         <v>8.51</v>
       </c>
       <c r="P2" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="Q2" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="R2">
         <v>14.505273478215095</v>
@@ -1563,10 +1682,10 @@
         <v>8.51</v>
       </c>
       <c r="P3" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="Q3" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="R3">
         <v>14.505273478215095</v>
@@ -1766,10 +1885,10 @@
         <v>8.49</v>
       </c>
       <c r="P4" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="Q4" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="R4">
         <v>14.272444048388209</v>
@@ -1960,10 +2079,10 @@
         <v>8.4700000000000006</v>
       </c>
       <c r="P5" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="Q5" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="R5">
         <v>11.105963802742538</v>
@@ -2206,7 +2325,7 @@
         <v>132</v>
       </c>
       <c r="C8" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D8" t="s">
         <v>137</v>
@@ -2247,6 +2366,450 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A639DD45-9E41-4F98-B389-5C28F46CFA6A}">
+  <dimension ref="A1:D31"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="16" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B2">
+        <v>2016</v>
+      </c>
+      <c r="C2" s="10">
+        <v>0.29481154500000001</v>
+      </c>
+      <c r="D2">
+        <v>0.51570487399999998</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="16" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B3">
+        <v>2017</v>
+      </c>
+      <c r="C3" s="10">
+        <v>1.8343823299999999</v>
+      </c>
+      <c r="D3">
+        <v>4.5747545680000004</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="16" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>62</v>
+      </c>
+      <c r="B4">
+        <v>2018</v>
+      </c>
+      <c r="C4" s="10">
+        <v>0.299537</v>
+      </c>
+      <c r="D4">
+        <v>2.1201708369999999</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="16" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>62</v>
+      </c>
+      <c r="B5">
+        <v>2019</v>
+      </c>
+      <c r="C5" s="10">
+        <v>0.24527299999999999</v>
+      </c>
+      <c r="D5">
+        <v>0.51302409900000001</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="16" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>62</v>
+      </c>
+      <c r="B6">
+        <v>2020</v>
+      </c>
+      <c r="C6" s="10">
+        <v>1.5348229200000001</v>
+      </c>
+      <c r="D6">
+        <v>2.4939214089999999</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>62</v>
+      </c>
+      <c r="B7">
+        <v>2021</v>
+      </c>
+      <c r="C7">
+        <v>0.69021067999999997</v>
+      </c>
+      <c r="D7">
+        <v>0.85490321700000005</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="16" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>107</v>
+      </c>
+      <c r="B8">
+        <v>2016</v>
+      </c>
+      <c r="C8" s="10">
+        <v>6.9886700000000004E-4</v>
+      </c>
+      <c r="D8">
+        <v>1.4843695000000001E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="16" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>107</v>
+      </c>
+      <c r="B9">
+        <v>2017</v>
+      </c>
+      <c r="C9" s="10">
+        <v>6.3414999999999999E-4</v>
+      </c>
+      <c r="D9">
+        <v>1.3469181E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="16" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>107</v>
+      </c>
+      <c r="B10">
+        <v>2018</v>
+      </c>
+      <c r="C10" s="12">
+        <v>4.0599999999999998E-5</v>
+      </c>
+      <c r="D10">
+        <v>8.6192599999999995E-4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="16" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>107</v>
+      </c>
+      <c r="B11">
+        <v>2019</v>
+      </c>
+      <c r="C11" s="10">
+        <v>3.4200000000000002E-4</v>
+      </c>
+      <c r="D11">
+        <v>7.2614480000000002E-3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="16" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>107</v>
+      </c>
+      <c r="B12">
+        <v>2020</v>
+      </c>
+      <c r="C12" s="10">
+        <v>1.4584E-4</v>
+      </c>
+      <c r="D12">
+        <v>3.0975909999999998E-3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>107</v>
+      </c>
+      <c r="B13">
+        <v>2021</v>
+      </c>
+      <c r="C13">
+        <v>6.6331599999999995E-4</v>
+      </c>
+      <c r="D13">
+        <v>1.4088623E-2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="16" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>108</v>
+      </c>
+      <c r="B14">
+        <v>2016</v>
+      </c>
+      <c r="C14" s="10">
+        <v>0.15317381499999999</v>
+      </c>
+      <c r="D14">
+        <v>0.100803244</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="16" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>108</v>
+      </c>
+      <c r="B15">
+        <v>2017</v>
+      </c>
+      <c r="C15" s="10">
+        <v>0.17322140999999999</v>
+      </c>
+      <c r="D15">
+        <v>5.3227802999999997E-2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="16" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>108</v>
+      </c>
+      <c r="B16">
+        <v>2018</v>
+      </c>
+      <c r="C16" s="10">
+        <v>0.124649</v>
+      </c>
+      <c r="D16">
+        <v>3.0795511000000001E-2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="16" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>108</v>
+      </c>
+      <c r="B17">
+        <v>2019</v>
+      </c>
+      <c r="C17" s="10">
+        <v>0.23880899999999999</v>
+      </c>
+      <c r="D17">
+        <v>5.4198745999999999E-2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="16" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>108</v>
+      </c>
+      <c r="B18">
+        <v>2020</v>
+      </c>
+      <c r="C18" s="10">
+        <v>0.114981425</v>
+      </c>
+      <c r="D18">
+        <v>4.9459030000000001E-2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>108</v>
+      </c>
+      <c r="B19">
+        <v>2021</v>
+      </c>
+      <c r="C19">
+        <v>0.16141213200000001</v>
+      </c>
+      <c r="D19">
+        <v>0.18539002800000001</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="16" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>20</v>
+      </c>
+      <c r="B20">
+        <v>2016</v>
+      </c>
+      <c r="C20" s="10">
+        <v>2.9962447559999998</v>
+      </c>
+      <c r="D20">
+        <v>12.975733419999999</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="16" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>20</v>
+      </c>
+      <c r="B21">
+        <v>2017</v>
+      </c>
+      <c r="C21" s="10">
+        <v>4.0498032899999998</v>
+      </c>
+      <c r="D21">
+        <v>10.91386782</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="16" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>20</v>
+      </c>
+      <c r="B22">
+        <v>2018</v>
+      </c>
+      <c r="C22" s="10">
+        <v>3.928868</v>
+      </c>
+      <c r="D22">
+        <v>11.437614030000001</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="16" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>20</v>
+      </c>
+      <c r="B23">
+        <v>2019</v>
+      </c>
+      <c r="C23" s="10">
+        <v>2.4504079999999999</v>
+      </c>
+      <c r="D23">
+        <v>7.5853045139999997</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="16" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>20</v>
+      </c>
+      <c r="B24">
+        <v>2020</v>
+      </c>
+      <c r="C24" s="10">
+        <v>3.9996879010000002</v>
+      </c>
+      <c r="D24">
+        <v>3.9139286740000001</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>20</v>
+      </c>
+      <c r="B25">
+        <v>2021</v>
+      </c>
+      <c r="C25">
+        <v>4.1384511689999997</v>
+      </c>
+      <c r="D25">
+        <v>24.036114179999998</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" ht="16" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>26</v>
+      </c>
+      <c r="B26">
+        <v>2016</v>
+      </c>
+      <c r="C26" s="10">
+        <v>6.382081157</v>
+      </c>
+      <c r="D26" s="11">
+        <v>46.048534119999999</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" ht="16" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>26</v>
+      </c>
+      <c r="B27">
+        <v>2017</v>
+      </c>
+      <c r="C27" s="10">
+        <v>5.3030500800000002</v>
+      </c>
+      <c r="D27" s="11">
+        <v>46.732286799999997</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" ht="16" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>26</v>
+      </c>
+      <c r="B28">
+        <v>2018</v>
+      </c>
+      <c r="C28" s="10">
+        <v>2.5902370000000001</v>
+      </c>
+      <c r="D28" s="11">
+        <v>35.544879999999999</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" ht="16" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>26</v>
+      </c>
+      <c r="B29">
+        <v>2019</v>
+      </c>
+      <c r="C29" s="10">
+        <v>1.112557</v>
+      </c>
+      <c r="D29" s="11">
+        <v>29.33484</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" ht="16" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>26</v>
+      </c>
+      <c r="B30">
+        <v>2020</v>
+      </c>
+      <c r="C30" s="10">
+        <v>1.8527943440000001</v>
+      </c>
+      <c r="D30" s="11">
+        <v>91.386446129999996</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>26</v>
+      </c>
+      <c r="B31">
+        <v>2021</v>
+      </c>
+      <c r="C31">
+        <v>10.3817766</v>
+      </c>
+      <c r="D31">
+        <v>52.646818469999999</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1CD37BC-78DE-4393-BD94-8F05FF676FE1}">
   <sheetPr filterMode="1"/>
   <dimension ref="A1:L160"/>
@@ -8152,357 +8715,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A639DD45-9E41-4F98-B389-5C28F46CFA6A}">
-  <dimension ref="A1:C31"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A1" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>153</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>62</v>
-      </c>
-      <c r="B2">
-        <v>0.51570487399999998</v>
-      </c>
-      <c r="C2">
-        <v>2016</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>62</v>
-      </c>
-      <c r="B3">
-        <v>4.5747545680000004</v>
-      </c>
-      <c r="C3">
-        <v>2017</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>62</v>
-      </c>
-      <c r="B4">
-        <v>2.1201708369999999</v>
-      </c>
-      <c r="C4">
-        <v>2018</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>62</v>
-      </c>
-      <c r="B5">
-        <v>0.51302409900000001</v>
-      </c>
-      <c r="C5">
-        <v>2019</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>62</v>
-      </c>
-      <c r="B6">
-        <v>2.4939214089999999</v>
-      </c>
-      <c r="C6">
-        <v>2020</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>62</v>
-      </c>
-      <c r="B7">
-        <v>0.85490321700000005</v>
-      </c>
-      <c r="C7">
-        <v>2021</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
-        <v>107</v>
-      </c>
-      <c r="B8">
-        <v>1.4843695000000001E-2</v>
-      </c>
-      <c r="C8">
-        <v>2016</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>107</v>
-      </c>
-      <c r="B9">
-        <v>1.3469181E-2</v>
-      </c>
-      <c r="C9">
-        <v>2017</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
-        <v>107</v>
-      </c>
-      <c r="B10">
-        <v>8.6192599999999995E-4</v>
-      </c>
-      <c r="C10">
-        <v>2018</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
-        <v>107</v>
-      </c>
-      <c r="B11">
-        <v>7.2614480000000002E-3</v>
-      </c>
-      <c r="C11">
-        <v>2019</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
-        <v>107</v>
-      </c>
-      <c r="B12">
-        <v>3.0975909999999998E-3</v>
-      </c>
-      <c r="C12">
-        <v>2020</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A13" t="s">
-        <v>107</v>
-      </c>
-      <c r="B13">
-        <v>1.4088623E-2</v>
-      </c>
-      <c r="C13">
-        <v>2021</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A14" t="s">
-        <v>108</v>
-      </c>
-      <c r="B14">
-        <v>0.100803244</v>
-      </c>
-      <c r="C14">
-        <v>2016</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A15" t="s">
-        <v>108</v>
-      </c>
-      <c r="B15">
-        <v>5.3227802999999997E-2</v>
-      </c>
-      <c r="C15">
-        <v>2017</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A16" t="s">
-        <v>108</v>
-      </c>
-      <c r="B16">
-        <v>3.0795511000000001E-2</v>
-      </c>
-      <c r="C16">
-        <v>2018</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A17" t="s">
-        <v>108</v>
-      </c>
-      <c r="B17">
-        <v>5.4198745999999999E-2</v>
-      </c>
-      <c r="C17">
-        <v>2019</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A18" t="s">
-        <v>108</v>
-      </c>
-      <c r="B18">
-        <v>4.9459030000000001E-2</v>
-      </c>
-      <c r="C18">
-        <v>2020</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A19" t="s">
-        <v>108</v>
-      </c>
-      <c r="B19">
-        <v>0.18539002800000001</v>
-      </c>
-      <c r="C19">
-        <v>2021</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A20" t="s">
-        <v>20</v>
-      </c>
-      <c r="B20">
-        <v>12.975733419999999</v>
-      </c>
-      <c r="C20">
-        <v>2016</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A21" t="s">
-        <v>20</v>
-      </c>
-      <c r="B21">
-        <v>10.91386782</v>
-      </c>
-      <c r="C21">
-        <v>2017</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A22" t="s">
-        <v>20</v>
-      </c>
-      <c r="B22">
-        <v>11.437614030000001</v>
-      </c>
-      <c r="C22">
-        <v>2018</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A23" t="s">
-        <v>20</v>
-      </c>
-      <c r="B23">
-        <v>7.5853045139999997</v>
-      </c>
-      <c r="C23">
-        <v>2019</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A24" t="s">
-        <v>20</v>
-      </c>
-      <c r="B24">
-        <v>3.9139286740000001</v>
-      </c>
-      <c r="C24">
-        <v>2020</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A25" t="s">
-        <v>20</v>
-      </c>
-      <c r="B25">
-        <v>24.036114179999998</v>
-      </c>
-      <c r="C25">
-        <v>2021</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A26" t="s">
-        <v>26</v>
-      </c>
-      <c r="B26">
-        <v>1.8622407329999999</v>
-      </c>
-      <c r="C26">
-        <v>2016</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A27" t="s">
-        <v>26</v>
-      </c>
-      <c r="B27">
-        <v>1.607085976</v>
-      </c>
-      <c r="C27">
-        <v>2017</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A28" t="s">
-        <v>26</v>
-      </c>
-      <c r="B28">
-        <v>2.98806561</v>
-      </c>
-      <c r="C28">
-        <v>2018</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A29" t="s">
-        <v>26</v>
-      </c>
-      <c r="B29">
-        <v>2.6448402579999999</v>
-      </c>
-      <c r="C29">
-        <v>2019</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A30" t="s">
-        <v>26</v>
-      </c>
-      <c r="B30">
-        <v>1.893528774</v>
-      </c>
-      <c r="C30">
-        <v>2020</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A31" t="s">
-        <v>26</v>
-      </c>
-      <c r="B31">
-        <v>5.036572853</v>
-      </c>
-      <c r="C31">
-        <v>2021</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1DD69A6-9758-46F5-A03C-8A6B27428E10}">
   <dimension ref="A1:D9"/>
@@ -8513,13 +8725,13 @@
         <v>152</v>
       </c>
       <c r="B1" t="s">
+        <v>214</v>
+      </c>
+      <c r="C1" t="s">
         <v>215</v>
       </c>
-      <c r="C1" t="s">
-        <v>216</v>
-      </c>
       <c r="D1" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
@@ -8531,7 +8743,7 @@
         <v>312.5</v>
       </c>
       <c r="C2" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
@@ -8543,7 +8755,7 @@
         <v>430.5555555555556</v>
       </c>
       <c r="C3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
@@ -8555,7 +8767,7 @@
         <v>194.44444444444443</v>
       </c>
       <c r="C4" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
@@ -8567,7 +8779,7 @@
         <v>361.11111111111109</v>
       </c>
       <c r="C5" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
@@ -8579,7 +8791,7 @@
         <v>652.77777777777783</v>
       </c>
       <c r="C6" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
@@ -8591,7 +8803,7 @@
         <v>381.9444444444444</v>
       </c>
       <c r="C7" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
@@ -8603,7 +8815,7 @@
         <v>277.77777777777777</v>
       </c>
       <c r="C8" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
@@ -8615,7 +8827,7 @@
         <v>180.55555555555554</v>
       </c>
       <c r="C9" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
   </sheetData>
@@ -8624,190 +8836,188 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C1934CC-AF7C-4B16-A1BA-6A4CD2D5F7CF}">
-  <dimension ref="A1:F12"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{984CFD00-4649-4709-AB3C-2647697CD4C9}">
+  <dimension ref="A1:F9"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
+      <c r="A1" s="13" t="s">
         <v>152</v>
       </c>
-      <c r="B1" t="s">
-        <v>153</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="13" t="s">
+        <v>220</v>
+      </c>
+      <c r="C1" s="13" t="s">
+        <v>245</v>
+      </c>
+      <c r="D1" s="13" t="s">
+        <v>247</v>
+      </c>
+      <c r="E1" s="13" t="s">
+        <v>248</v>
+      </c>
+      <c r="F1" s="13" t="s">
         <v>215</v>
       </c>
-      <c r="D1" t="s">
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>221</v>
       </c>
-      <c r="E1" t="s">
+      <c r="B2">
+        <v>47</v>
+      </c>
+      <c r="C2">
+        <v>186.04651162790691</v>
+      </c>
+      <c r="D2">
+        <v>478.30148374891041</v>
+      </c>
+      <c r="E2">
+        <v>69.767441860465169</v>
+      </c>
+      <c r="F2" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
         <v>222</v>
       </c>
-      <c r="F1" t="s">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A2">
-        <v>2020</v>
-      </c>
-      <c r="B2">
-        <v>99</v>
-      </c>
-      <c r="D2">
-        <v>117</v>
-      </c>
-      <c r="F2" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A3">
-        <v>2019</v>
-      </c>
       <c r="B3">
-        <f>AVERAGE(136,96)</f>
-        <v>116</v>
+        <v>37</v>
+      </c>
+      <c r="C3">
+        <v>279.06976744186028</v>
       </c>
       <c r="D3">
-        <f>AVERAGE(108,102)</f>
-        <v>105</v>
+        <v>353.64898431966373</v>
+      </c>
+      <c r="E3">
+        <v>58.139534883720899</v>
       </c>
       <c r="F3" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A4">
-        <v>2018</v>
+      <c r="A4" t="s">
+        <v>223</v>
       </c>
       <c r="B4">
-        <v>88</v>
+        <v>30</v>
+      </c>
+      <c r="C4">
+        <v>383.72093023255809</v>
       </c>
       <c r="D4">
-        <v>52</v>
+        <v>636.88669477344922</v>
+      </c>
+      <c r="E4">
+        <v>116.2790697674419</v>
       </c>
       <c r="F4" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A5">
-        <v>2017</v>
+      <c r="A5" t="s">
+        <v>224</v>
       </c>
       <c r="B5">
-        <f>AVERAGE(96,46)</f>
-        <v>71</v>
+        <v>107</v>
+      </c>
+      <c r="C5">
+        <v>662.79069767441854</v>
       </c>
       <c r="D5">
-        <f>AVERAGE(69,43)</f>
-        <v>56</v>
+        <v>2044.760085551236</v>
+      </c>
+      <c r="E5">
+        <v>197.67441860465121</v>
       </c>
       <c r="F5" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A6">
-        <v>2016</v>
+      <c r="A6" t="s">
+        <v>228</v>
       </c>
       <c r="B6">
-        <f>AVERAGE(101, 74)</f>
-        <v>87.5</v>
+        <v>283</v>
+      </c>
+      <c r="C6">
+        <v>358.1850316138665</v>
       </c>
       <c r="D6">
-        <f>AVERAGE(75, 57)</f>
-        <v>66</v>
+        <v>1022.580213060133</v>
+      </c>
+      <c r="E6">
+        <v>60.786084170397878</v>
       </c>
       <c r="F6" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A7">
-        <v>2015</v>
+      <c r="A7" t="s">
+        <v>225</v>
       </c>
       <c r="B7">
-        <f>AVERAGE(122, 86)</f>
-        <v>104</v>
+        <v>135</v>
+      </c>
+      <c r="C7">
+        <v>197.67441860465101</v>
       </c>
       <c r="D7">
-        <f>AVERAGE(100, 66)</f>
-        <v>83</v>
+        <v>405.31221064961238</v>
+      </c>
+      <c r="E7">
+        <v>34.883720930232471</v>
       </c>
       <c r="F7" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A8">
-        <v>2014</v>
+      <c r="A8" t="s">
+        <v>226</v>
       </c>
       <c r="B8">
-        <f>AVERAGE(194, 178)</f>
-        <v>186</v>
+        <v>107</v>
+      </c>
+      <c r="C8">
+        <v>441.86046511627899</v>
       </c>
       <c r="D8">
-        <f>AVERAGE(173, 113)</f>
-        <v>143</v>
+        <v>601.40002516212769</v>
+      </c>
+      <c r="E8">
+        <v>58.139534883720899</v>
       </c>
       <c r="F8" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A9">
-        <v>2013</v>
+      <c r="A9" t="s">
+        <v>227</v>
       </c>
       <c r="B9">
-        <f>AVERAGE(310, 235)</f>
-        <v>272.5</v>
+        <v>93</v>
+      </c>
+      <c r="C9">
+        <v>313.95348837209281</v>
       </c>
       <c r="D9">
-        <f>AVERAGE(249, 154)</f>
-        <v>201.5</v>
+        <v>784.9483177552396</v>
+      </c>
+      <c r="E9">
+        <v>81.395348837209212</v>
       </c>
       <c r="F9" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A10">
-        <v>2019</v>
-      </c>
-      <c r="C10">
-        <v>48</v>
-      </c>
-      <c r="E10">
-        <v>19.600000000000001</v>
-      </c>
-      <c r="F10" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A11">
-        <v>2014</v>
-      </c>
-      <c r="C11">
-        <f>1.6/3.2*500</f>
-        <v>250</v>
-      </c>
-      <c r="F11" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A12">
-        <v>2011</v>
-      </c>
-      <c r="C12">
-        <f>2.7/3.2*500</f>
-        <v>421.875</v>
-      </c>
-      <c r="F12" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
     </row>
   </sheetData>
@@ -8816,6 +9026,595 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{40C4BB59-8C51-4F8F-8B75-11BF228EC6E5}">
+  <dimension ref="A1:P9"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>152</v>
+      </c>
+      <c r="B1" t="s">
+        <v>230</v>
+      </c>
+      <c r="C1" t="s">
+        <v>231</v>
+      </c>
+      <c r="D1" t="s">
+        <v>233</v>
+      </c>
+      <c r="E1" t="s">
+        <v>234</v>
+      </c>
+      <c r="F1" t="s">
+        <v>240</v>
+      </c>
+      <c r="G1" t="s">
+        <v>235</v>
+      </c>
+      <c r="H1" t="s">
+        <v>236</v>
+      </c>
+      <c r="I1" t="s">
+        <v>237</v>
+      </c>
+      <c r="J1" t="s">
+        <v>238</v>
+      </c>
+      <c r="K1" t="s">
+        <v>239</v>
+      </c>
+      <c r="P1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>2013</v>
+      </c>
+      <c r="B2">
+        <v>41</v>
+      </c>
+      <c r="C2">
+        <v>41</v>
+      </c>
+      <c r="D2">
+        <v>156.5</v>
+      </c>
+      <c r="E2">
+        <v>117.6</v>
+      </c>
+      <c r="F2">
+        <f>AVERAGE(D2:E2)</f>
+        <v>137.05000000000001</v>
+      </c>
+      <c r="G2">
+        <v>19.600000000000001</v>
+      </c>
+      <c r="H2">
+        <v>12.1</v>
+      </c>
+      <c r="I2">
+        <f>G2*SQRT(B2)</f>
+        <v>125.50123505368384</v>
+      </c>
+      <c r="J2">
+        <f>H2*SQRT(C2)</f>
+        <v>77.477803272937464</v>
+      </c>
+      <c r="K2">
+        <f>SQRT(((B2-1)*I2^2+(C2-1)*J2^2)/(B2+C2-2))</f>
+        <v>104.29134671678183</v>
+      </c>
+      <c r="P2" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>2014</v>
+      </c>
+      <c r="B3">
+        <v>41</v>
+      </c>
+      <c r="C3">
+        <v>41</v>
+      </c>
+      <c r="D3">
+        <v>97.8</v>
+      </c>
+      <c r="E3">
+        <v>89</v>
+      </c>
+      <c r="F3">
+        <f t="shared" ref="F3:F9" si="0">AVERAGE(D3:E3)</f>
+        <v>93.4</v>
+      </c>
+      <c r="G3">
+        <v>13.5</v>
+      </c>
+      <c r="H3">
+        <v>8.8000000000000007</v>
+      </c>
+      <c r="I3">
+        <f t="shared" ref="I3:I9" si="1">G3*SQRT(B3)</f>
+        <v>86.442177205343455</v>
+      </c>
+      <c r="J3">
+        <f t="shared" ref="J3:J9" si="2">H3*SQRT(C3)</f>
+        <v>56.347493289409073</v>
+      </c>
+      <c r="K3">
+        <f t="shared" ref="K3:K9" si="3">SQRT(((B3-1)*I3^2+(C3-1)*J3^2)/(B3+C3-2))</f>
+        <v>72.963312698917392</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A4">
+        <v>2015</v>
+      </c>
+      <c r="B4">
+        <v>41</v>
+      </c>
+      <c r="C4">
+        <v>41</v>
+      </c>
+      <c r="D4">
+        <v>61.7</v>
+      </c>
+      <c r="E4">
+        <v>43.3</v>
+      </c>
+      <c r="F4">
+        <f t="shared" si="0"/>
+        <v>52.5</v>
+      </c>
+      <c r="G4">
+        <v>7.9</v>
+      </c>
+      <c r="H4">
+        <v>5.2</v>
+      </c>
+      <c r="I4">
+        <f t="shared" si="1"/>
+        <v>50.584681475719506</v>
+      </c>
+      <c r="J4">
+        <f t="shared" si="2"/>
+        <v>33.296246034650814</v>
+      </c>
+      <c r="K4">
+        <f t="shared" si="3"/>
+        <v>42.822015365930639</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>2016</v>
+      </c>
+      <c r="B5">
+        <v>41</v>
+      </c>
+      <c r="C5">
+        <v>41</v>
+      </c>
+      <c r="D5">
+        <v>51.9</v>
+      </c>
+      <c r="E5">
+        <v>36.9</v>
+      </c>
+      <c r="F5">
+        <f t="shared" si="0"/>
+        <v>44.4</v>
+      </c>
+      <c r="G5">
+        <v>6.2</v>
+      </c>
+      <c r="H5">
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="I5">
+        <f>G5*SQRT(B5)</f>
+        <v>39.699370272083662</v>
+      </c>
+      <c r="J5">
+        <f t="shared" si="2"/>
+        <v>28.173746644704536</v>
+      </c>
+      <c r="K5">
+        <f t="shared" si="3"/>
+        <v>34.4223764432382</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>2017</v>
+      </c>
+      <c r="B6">
+        <v>36</v>
+      </c>
+      <c r="C6">
+        <v>41</v>
+      </c>
+      <c r="D6">
+        <v>47.8</v>
+      </c>
+      <c r="E6">
+        <v>22.8</v>
+      </c>
+      <c r="F6">
+        <f t="shared" si="0"/>
+        <v>35.299999999999997</v>
+      </c>
+      <c r="G6">
+        <v>5.8</v>
+      </c>
+      <c r="H6">
+        <v>3.4</v>
+      </c>
+      <c r="I6">
+        <f t="shared" si="1"/>
+        <v>34.799999999999997</v>
+      </c>
+      <c r="J6">
+        <f t="shared" si="2"/>
+        <v>21.770622407271684</v>
+      </c>
+      <c r="K6">
+        <f t="shared" si="3"/>
+        <v>28.599487174889457</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A7">
+        <v>2018</v>
+      </c>
+      <c r="C7">
+        <v>41</v>
+      </c>
+      <c r="E7">
+        <v>44.3</v>
+      </c>
+      <c r="F7">
+        <f t="shared" si="0"/>
+        <v>44.3</v>
+      </c>
+      <c r="H7">
+        <v>4</v>
+      </c>
+      <c r="I7">
+        <f>G7*SQRT(B5)</f>
+        <v>0</v>
+      </c>
+      <c r="J7">
+        <f t="shared" si="2"/>
+        <v>25.612496949731394</v>
+      </c>
+      <c r="K7">
+        <f t="shared" si="3"/>
+        <v>25.938783950303314</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A8">
+        <v>2019</v>
+      </c>
+      <c r="B8">
+        <v>41</v>
+      </c>
+      <c r="C8">
+        <v>41</v>
+      </c>
+      <c r="D8">
+        <v>65</v>
+      </c>
+      <c r="E8">
+        <v>48</v>
+      </c>
+      <c r="F8">
+        <f t="shared" si="0"/>
+        <v>56.5</v>
+      </c>
+      <c r="G8">
+        <v>8.9</v>
+      </c>
+      <c r="H8">
+        <v>8</v>
+      </c>
+      <c r="I8">
+        <f t="shared" si="1"/>
+        <v>56.987805713152355</v>
+      </c>
+      <c r="J8">
+        <f t="shared" si="2"/>
+        <v>51.224993899462788</v>
+      </c>
+      <c r="K8">
+        <f t="shared" si="3"/>
+        <v>54.183069311363305</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A9">
+        <v>2020</v>
+      </c>
+      <c r="C9">
+        <v>26</v>
+      </c>
+      <c r="E9">
+        <v>49.4</v>
+      </c>
+      <c r="F9">
+        <f t="shared" si="0"/>
+        <v>49.4</v>
+      </c>
+      <c r="H9">
+        <v>11.5</v>
+      </c>
+      <c r="I9">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J9">
+        <f t="shared" si="2"/>
+        <v>58.638724406317024</v>
+      </c>
+      <c r="K9">
+        <f t="shared" si="3"/>
+        <v>59.84789748465132</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C1934CC-AF7C-4B16-A1BA-6A4CD2D5F7CF}">
+  <dimension ref="A1:I12"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>152</v>
+      </c>
+      <c r="B1" t="s">
+        <v>241</v>
+      </c>
+      <c r="C1" t="s">
+        <v>242</v>
+      </c>
+      <c r="D1" t="s">
+        <v>243</v>
+      </c>
+      <c r="E1" t="s">
+        <v>244</v>
+      </c>
+      <c r="F1" t="s">
+        <v>245</v>
+      </c>
+      <c r="G1" t="s">
+        <v>246</v>
+      </c>
+      <c r="H1" t="s">
+        <v>247</v>
+      </c>
+      <c r="I1" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>2013</v>
+      </c>
+      <c r="C2">
+        <v>41</v>
+      </c>
+      <c r="D2">
+        <v>41</v>
+      </c>
+      <c r="E2">
+        <v>137.05000000000001</v>
+      </c>
+      <c r="G2">
+        <v>104.29134670000001</v>
+      </c>
+      <c r="I2" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>2014</v>
+      </c>
+      <c r="C3">
+        <v>41</v>
+      </c>
+      <c r="D3">
+        <v>41</v>
+      </c>
+      <c r="E3">
+        <v>93.4</v>
+      </c>
+      <c r="G3">
+        <v>72.963312700000003</v>
+      </c>
+      <c r="I3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A4">
+        <v>2015</v>
+      </c>
+      <c r="C4">
+        <v>41</v>
+      </c>
+      <c r="D4">
+        <v>41</v>
+      </c>
+      <c r="E4">
+        <v>52.5</v>
+      </c>
+      <c r="G4">
+        <v>42.822015370000003</v>
+      </c>
+      <c r="I4" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>2016</v>
+      </c>
+      <c r="C5">
+        <v>41</v>
+      </c>
+      <c r="D5">
+        <v>41</v>
+      </c>
+      <c r="E5">
+        <v>44.4</v>
+      </c>
+      <c r="G5">
+        <v>34.422376440000001</v>
+      </c>
+      <c r="I5" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>2017</v>
+      </c>
+      <c r="C6">
+        <v>36</v>
+      </c>
+      <c r="D6">
+        <v>41</v>
+      </c>
+      <c r="E6">
+        <v>35.299999999999997</v>
+      </c>
+      <c r="G6">
+        <v>28.59948717</v>
+      </c>
+      <c r="I6" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A7">
+        <v>2018</v>
+      </c>
+      <c r="D7">
+        <v>41</v>
+      </c>
+      <c r="E7">
+        <v>44.3</v>
+      </c>
+      <c r="G7">
+        <v>25.938783950000001</v>
+      </c>
+      <c r="I7" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A8">
+        <v>2019</v>
+      </c>
+      <c r="C8">
+        <v>41</v>
+      </c>
+      <c r="D8">
+        <v>41</v>
+      </c>
+      <c r="E8">
+        <v>56.5</v>
+      </c>
+      <c r="G8">
+        <v>54.18306931</v>
+      </c>
+      <c r="I8" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A9">
+        <v>2020</v>
+      </c>
+      <c r="D9">
+        <v>26</v>
+      </c>
+      <c r="E9">
+        <v>49.4</v>
+      </c>
+      <c r="G9">
+        <v>59.84789748</v>
+      </c>
+      <c r="I9" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A10">
+        <v>2011</v>
+      </c>
+      <c r="B10">
+        <v>18</v>
+      </c>
+      <c r="F10">
+        <v>410.52631580000002</v>
+      </c>
+      <c r="H10">
+        <v>164.0890239</v>
+      </c>
+      <c r="I10" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A11">
+        <v>2014</v>
+      </c>
+      <c r="B11">
+        <v>22</v>
+      </c>
+      <c r="F11">
+        <v>242.1052632</v>
+      </c>
+      <c r="H11">
+        <v>444.35517720000001</v>
+      </c>
+      <c r="I11" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A12">
+        <v>2019</v>
+      </c>
+      <c r="B12">
+        <v>27</v>
+      </c>
+      <c r="F12">
+        <v>48.271646859999997</v>
+      </c>
+      <c r="H12">
+        <v>179.02166930000001</v>
+      </c>
+      <c r="I12" t="s">
+        <v>250</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCB797C5-CB47-4805-AD51-BAF5F7220E5D}">
   <dimension ref="A1:AF17"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -9060,10 +9859,10 @@
         <v>151</v>
       </c>
       <c r="AE17" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="AF17" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
   </sheetData>
@@ -9072,7 +9871,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4782880F-19F5-4C97-B687-8149361B0730}">
   <dimension ref="A1:CJ160"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -9151,13 +9950,13 @@
         <v>99</v>
       </c>
       <c r="Y1" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="Z1" s="3" t="s">
         <v>156</v>
       </c>
-      <c r="Z1" s="3" t="s">
+      <c r="AA1" s="3" t="s">
         <v>157</v>
-      </c>
-      <c r="AA1" s="3" t="s">
-        <v>158</v>
       </c>
       <c r="AB1" s="3" t="s">
         <v>146</v>
@@ -9187,160 +9986,160 @@
         <v>5</v>
       </c>
       <c r="AK1" t="s">
+        <v>158</v>
+      </c>
+      <c r="AL1" t="s">
         <v>159</v>
-      </c>
-      <c r="AL1" t="s">
-        <v>160</v>
       </c>
       <c r="AM1" t="s">
         <v>97</v>
       </c>
       <c r="AN1" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="AO1" t="s">
+        <v>160</v>
+      </c>
+      <c r="AP1" t="s">
         <v>161</v>
       </c>
-      <c r="AP1" t="s">
+      <c r="AQ1" t="s">
         <v>162</v>
       </c>
-      <c r="AQ1" t="s">
+      <c r="AR1" t="s">
         <v>163</v>
       </c>
-      <c r="AR1" t="s">
+      <c r="AS1" t="s">
         <v>164</v>
       </c>
-      <c r="AS1" t="s">
+      <c r="AT1" t="s">
         <v>165</v>
       </c>
-      <c r="AT1" t="s">
+      <c r="AU1" t="s">
         <v>166</v>
       </c>
-      <c r="AU1" t="s">
+      <c r="AV1" t="s">
         <v>167</v>
       </c>
-      <c r="AV1" t="s">
+      <c r="AW1" t="s">
         <v>168</v>
       </c>
-      <c r="AW1" t="s">
+      <c r="AX1" t="s">
         <v>169</v>
       </c>
-      <c r="AX1" t="s">
+      <c r="AY1" t="s">
         <v>170</v>
       </c>
-      <c r="AY1" t="s">
+      <c r="AZ1" t="s">
         <v>171</v>
       </c>
-      <c r="AZ1" t="s">
+      <c r="BA1" t="s">
         <v>172</v>
       </c>
-      <c r="BA1" t="s">
+      <c r="BB1" t="s">
         <v>173</v>
       </c>
-      <c r="BB1" t="s">
+      <c r="BC1" t="s">
         <v>174</v>
       </c>
-      <c r="BC1" t="s">
+      <c r="BD1" t="s">
         <v>175</v>
       </c>
-      <c r="BD1" t="s">
+      <c r="BE1" t="s">
         <v>176</v>
       </c>
-      <c r="BE1" t="s">
+      <c r="BF1" t="s">
         <v>177</v>
       </c>
-      <c r="BF1" t="s">
+      <c r="BG1" t="s">
         <v>178</v>
       </c>
-      <c r="BG1" t="s">
+      <c r="BH1" t="s">
         <v>179</v>
       </c>
-      <c r="BH1" t="s">
+      <c r="BI1" t="s">
         <v>180</v>
       </c>
-      <c r="BI1" t="s">
+      <c r="BJ1" t="s">
         <v>181</v>
       </c>
-      <c r="BJ1" t="s">
+      <c r="BK1" t="s">
         <v>182</v>
       </c>
-      <c r="BK1" t="s">
+      <c r="BL1" t="s">
         <v>183</v>
       </c>
-      <c r="BL1" t="s">
+      <c r="BM1" t="s">
         <v>184</v>
       </c>
-      <c r="BM1" t="s">
+      <c r="BN1" t="s">
         <v>185</v>
       </c>
-      <c r="BN1" t="s">
+      <c r="BO1" t="s">
         <v>186</v>
       </c>
-      <c r="BO1" t="s">
+      <c r="BP1" t="s">
         <v>187</v>
       </c>
-      <c r="BP1" t="s">
+      <c r="BQ1" t="s">
         <v>188</v>
       </c>
-      <c r="BQ1" t="s">
+      <c r="BR1" t="s">
         <v>189</v>
       </c>
-      <c r="BR1" t="s">
+      <c r="BS1" t="s">
         <v>190</v>
       </c>
-      <c r="BS1" t="s">
+      <c r="BT1" t="s">
         <v>191</v>
       </c>
-      <c r="BT1" t="s">
+      <c r="BU1" t="s">
         <v>192</v>
       </c>
-      <c r="BU1" t="s">
+      <c r="BV1" t="s">
         <v>193</v>
       </c>
-      <c r="BV1" t="s">
+      <c r="BW1" t="s">
         <v>194</v>
       </c>
-      <c r="BW1" t="s">
+      <c r="BX1" t="s">
         <v>195</v>
       </c>
-      <c r="BX1" t="s">
+      <c r="BY1" t="s">
         <v>196</v>
       </c>
-      <c r="BY1" t="s">
+      <c r="BZ1" t="s">
         <v>197</v>
       </c>
-      <c r="BZ1" t="s">
+      <c r="CA1" t="s">
         <v>198</v>
       </c>
-      <c r="CA1" t="s">
+      <c r="CB1" t="s">
         <v>199</v>
       </c>
-      <c r="CB1" t="s">
+      <c r="CC1" t="s">
         <v>200</v>
       </c>
-      <c r="CC1" t="s">
+      <c r="CD1" t="s">
         <v>201</v>
       </c>
-      <c r="CD1" t="s">
+      <c r="CE1" t="s">
         <v>202</v>
       </c>
-      <c r="CE1" t="s">
+      <c r="CF1" t="s">
         <v>203</v>
       </c>
-      <c r="CF1" t="s">
+      <c r="CG1" t="s">
         <v>204</v>
       </c>
-      <c r="CG1" t="s">
+      <c r="CH1" t="s">
         <v>205</v>
       </c>
-      <c r="CH1" t="s">
+      <c r="CI1" t="s">
         <v>206</v>
       </c>
-      <c r="CI1" t="s">
+      <c r="CJ1" t="s">
         <v>207</v>
-      </c>
-      <c r="CJ1" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="2" spans="1:88" x14ac:dyDescent="0.35">
@@ -9462,10 +10261,10 @@
         <v>8.51</v>
       </c>
       <c r="AK2" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AL2" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AM2" s="6">
         <v>14.505273478215095</v>
@@ -9737,10 +10536,10 @@
         <v>8.51</v>
       </c>
       <c r="AK3" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AL3" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AM3" s="6">
         <v>14.505273478215095</v>
@@ -10012,10 +10811,10 @@
         <v>8.51</v>
       </c>
       <c r="AK4" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AL4" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AM4" s="6">
         <v>14.505273478215095</v>
@@ -10287,10 +11086,10 @@
         <v>8.51</v>
       </c>
       <c r="AK5" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AL5" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AM5" s="6">
         <v>14.505273478215095</v>
@@ -10562,10 +11361,10 @@
         <v>8.51</v>
       </c>
       <c r="AK6" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AL6" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AM6" s="6">
         <v>14.505273478215095</v>
@@ -10837,10 +11636,10 @@
         <v>8.51</v>
       </c>
       <c r="AK7" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AL7" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AM7" s="6">
         <v>14.505273478215095</v>
@@ -11097,10 +11896,10 @@
         <v>8.51</v>
       </c>
       <c r="AK8" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AL8" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AM8" s="6">
         <v>14.505273478215095</v>
@@ -11357,10 +12156,10 @@
         <v>8.51</v>
       </c>
       <c r="AK9" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AL9" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AM9" s="6">
         <v>14.505273478215095</v>
@@ -11617,10 +12416,10 @@
         <v>8.51</v>
       </c>
       <c r="AK10" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AL10" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AM10" s="6">
         <v>14.505273478215095</v>
@@ -11877,10 +12676,10 @@
         <v>8.51</v>
       </c>
       <c r="AK11" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AL11" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AM11" s="6">
         <v>14.505273478215095</v>
@@ -12137,10 +12936,10 @@
         <v>8.51</v>
       </c>
       <c r="AK12" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AL12" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AM12" s="6">
         <v>14.505273478215095</v>
@@ -12397,10 +13196,10 @@
         <v>8.51</v>
       </c>
       <c r="AK13" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AL13" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AM13" s="6">
         <v>14.505273478215095</v>
@@ -12657,10 +13456,10 @@
         <v>8.51</v>
       </c>
       <c r="AK14" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AL14" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AM14" s="6">
         <v>14.505273478215095</v>
@@ -12917,10 +13716,10 @@
         <v>8.51</v>
       </c>
       <c r="AK15" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AL15" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AM15" s="6">
         <v>14.505273478215095</v>
@@ -13177,10 +13976,10 @@
         <v>8.51</v>
       </c>
       <c r="AK16" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AL16" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AM16" s="6">
         <v>14.505273478215095</v>
@@ -13437,10 +14236,10 @@
         <v>8.51</v>
       </c>
       <c r="AK17" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AL17" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AM17" s="6">
         <v>14.505273478215095</v>
@@ -13697,10 +14496,10 @@
         <v>8.51</v>
       </c>
       <c r="AK18" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AL18" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AM18" s="6">
         <v>14.505273478215095</v>
@@ -13957,10 +14756,10 @@
         <v>8.51</v>
       </c>
       <c r="AK19" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AL19" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AM19" s="6">
         <v>14.505273478215095</v>
@@ -14217,10 +15016,10 @@
         <v>8.51</v>
       </c>
       <c r="AK20" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AL20" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AM20" s="6">
         <v>14.505273478215095</v>
@@ -14477,10 +15276,10 @@
         <v>8.51</v>
       </c>
       <c r="AK21" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AL21" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AM21" s="6">
         <v>14.505273478215095</v>
@@ -14737,10 +15536,10 @@
         <v>8.51</v>
       </c>
       <c r="AK22" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AL22" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AM22" s="6">
         <v>14.505273478215095</v>
@@ -14997,10 +15796,10 @@
         <v>8.51</v>
       </c>
       <c r="AK23" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AL23" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AM23" s="6">
         <v>14.505273478215095</v>
@@ -15252,10 +16051,10 @@
         <v>8.51</v>
       </c>
       <c r="AK24" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AL24" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AM24" s="6">
         <v>14.505273478215095</v>
@@ -15507,10 +16306,10 @@
         <v>8.51</v>
       </c>
       <c r="AK25" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AL25" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AM25" s="6">
         <v>14.505273478215095</v>
@@ -15782,10 +16581,10 @@
         <v>8.49</v>
       </c>
       <c r="AK26" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AL26" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AM26" s="6">
         <v>14.272444048388209</v>
@@ -16058,10 +16857,10 @@
         <v>8.49</v>
       </c>
       <c r="AK27" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AL27" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AM27" s="6">
         <v>14.272444048388209</v>
@@ -16333,10 +17132,10 @@
         <v>8.49</v>
       </c>
       <c r="AK28" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AL28" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AM28" s="6">
         <v>14.272444048388209</v>
@@ -16608,10 +17407,10 @@
         <v>8.49</v>
       </c>
       <c r="AK29" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AL29" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AM29" s="6">
         <v>14.272444048388209</v>
@@ -16863,10 +17662,10 @@
         <v>8.49</v>
       </c>
       <c r="AK30" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AL30" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AM30" s="6">
         <v>14.272444048388209</v>
@@ -17138,10 +17937,10 @@
         <v>8.49</v>
       </c>
       <c r="AK31" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AL31" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AM31" s="6">
         <v>14.272444048388209</v>
@@ -17393,10 +18192,10 @@
         <v>8.49</v>
       </c>
       <c r="AK32" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AL32" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AM32" s="6">
         <v>14.272444048388209</v>
@@ -17668,10 +18467,10 @@
         <v>8.4700000000000006</v>
       </c>
       <c r="AK33" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AL33" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AM33">
         <v>11.105963802742538</v>
@@ -17943,10 +18742,10 @@
         <v>8.4700000000000006</v>
       </c>
       <c r="AK34" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AL34" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AM34">
         <v>11.105963802742538</v>
@@ -18218,10 +19017,10 @@
         <v>8.4700000000000006</v>
       </c>
       <c r="AK35" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AL35" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AM35">
         <v>11.105963802742538</v>
@@ -18493,10 +19292,10 @@
         <v>8.4700000000000006</v>
       </c>
       <c r="AK36" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AL36" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AM36">
         <v>11.105963802742538</v>
@@ -18768,10 +19567,10 @@
         <v>8.4700000000000006</v>
       </c>
       <c r="AK37" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AL37" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AM37">
         <v>11.105963802742538</v>
@@ -19028,10 +19827,10 @@
         <v>8.4700000000000006</v>
       </c>
       <c r="AK38" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AL38" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AM38">
         <v>11.105963802742538</v>
@@ -19303,10 +20102,10 @@
         <v>8.4700000000000006</v>
       </c>
       <c r="AK39" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AL39" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AM39">
         <v>11.105963802742538</v>
@@ -19578,10 +20377,10 @@
         <v>8.4700000000000006</v>
       </c>
       <c r="AK40" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AL40" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AM40">
         <v>11.105963802742538</v>
@@ -19841,10 +20640,10 @@
         <v>8.4700000000000006</v>
       </c>
       <c r="AK41" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AL41" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AM41">
         <v>11.105963802742538</v>
@@ -20117,10 +20916,10 @@
         <v>8.4700000000000006</v>
       </c>
       <c r="AK42" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AL42" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AM42">
         <v>11.105963802742538</v>
@@ -20372,10 +21171,10 @@
         <v>8.4700000000000006</v>
       </c>
       <c r="AK43" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AL43" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AM43">
         <v>11.105963802742538</v>
@@ -20648,10 +21447,10 @@
         <v>8.4700000000000006</v>
       </c>
       <c r="AK44" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AL44" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AM44">
         <v>11.105963802742538</v>
@@ -20924,10 +21723,10 @@
         <v>8.4700000000000006</v>
       </c>
       <c r="AK45" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AL45" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AM45">
         <v>11.105963802742538</v>
@@ -21200,10 +21999,10 @@
         <v>8.4700000000000006</v>
       </c>
       <c r="AK46" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AL46" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AM46">
         <v>11.105963802742538</v>
@@ -21455,10 +22254,10 @@
         <v>8.4700000000000006</v>
       </c>
       <c r="AK47" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AL47" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AM47">
         <v>11.105963802742538</v>
@@ -24530,7 +25329,7 @@
         <v>-927.026733972908</v>
       </c>
       <c r="AC73" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="AD73" t="s">
         <v>31</v>

</xml_diff>

<commit_message>
modified datasets, tables and figures for paper revisions R2
</commit_message>
<xml_diff>
--- a/data/2022-03-03_LakeErie_Mastersheet.xlsx
+++ b/data/2022-03-03_LakeErie_Mastersheet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://trentu-my.sharepoint.com/personal/sandraklemet_trentu_ca/Documents/Documents/Etudes/Trent/Xenopoulos lab/Projects/LakeErie_animal-excretion/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="817" documentId="13_ncr:1_{EA2E9A16-F367-47E5-9F32-F761EF32E94C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{912D02CB-F106-4F3B-B77D-F90FB25C016C}"/>
+  <xr:revisionPtr revIDLastSave="819" documentId="13_ncr:1_{EA2E9A16-F367-47E5-9F32-F761EF32E94C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{60046B3F-A6F4-4365-8EEB-6906EACACCF3}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="5" activeTab="6" xr2:uid="{FCD5901F-55C5-46A6-83E9-A175C073FB2F}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="5" activeTab="8" xr2:uid="{FCD5901F-55C5-46A6-83E9-A175C073FB2F}"/>
   </bookViews>
   <sheets>
     <sheet name="Fishing and Environmental data" sheetId="3" r:id="rId1"/>
@@ -22582,8 +22582,14 @@
       <c r="AI48" s="4">
         <v>8.3847586859687198</v>
       </c>
-    </row>
-    <row r="49" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="AM48">
+        <v>12.618307944649743</v>
+      </c>
+      <c r="AN48">
+        <v>1038.6948866828891</v>
+      </c>
+    </row>
+    <row r="49" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A49">
         <v>201</v>
       </c>
@@ -22699,8 +22705,14 @@
       <c r="AI49" s="4">
         <v>8.7270334952932984</v>
       </c>
-    </row>
-    <row r="50" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="AM49">
+        <v>12.618307944649743</v>
+      </c>
+      <c r="AN49">
+        <v>1038.6948866828891</v>
+      </c>
+    </row>
+    <row r="50" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A50">
         <v>202</v>
       </c>
@@ -22816,8 +22828,14 @@
       <c r="AI50" s="4">
         <v>9.1981531322659187</v>
       </c>
-    </row>
-    <row r="51" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="AM50">
+        <v>12.618307944649743</v>
+      </c>
+      <c r="AN50">
+        <v>1038.6948866828891</v>
+      </c>
+    </row>
+    <row r="51" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A51">
         <v>203</v>
       </c>
@@ -22933,8 +22951,14 @@
       <c r="AI51" s="4">
         <v>7.8831490516137386</v>
       </c>
-    </row>
-    <row r="52" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="AM51">
+        <v>12.618307944649743</v>
+      </c>
+      <c r="AN51">
+        <v>1038.6948866828891</v>
+      </c>
+    </row>
+    <row r="52" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A52">
         <v>204</v>
       </c>
@@ -23050,8 +23074,14 @@
       <c r="AI52" s="4">
         <v>7.8546261508366904</v>
       </c>
-    </row>
-    <row r="53" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="AM52">
+        <v>12.618307944649743</v>
+      </c>
+      <c r="AN52">
+        <v>1038.6948866828891</v>
+      </c>
+    </row>
+    <row r="53" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A53">
         <v>205</v>
       </c>
@@ -23165,8 +23195,14 @@
       <c r="AI53" s="4">
         <v>7.8438071195074652</v>
       </c>
-    </row>
-    <row r="54" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="AM53">
+        <v>12.618307944649743</v>
+      </c>
+      <c r="AN53">
+        <v>1038.6948866828891</v>
+      </c>
+    </row>
+    <row r="54" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A54">
         <v>206</v>
       </c>
@@ -23281,8 +23317,14 @@
       <c r="AI54" s="4">
         <v>9.9633537117329318</v>
       </c>
-    </row>
-    <row r="55" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="AM54">
+        <v>12.618307944649743</v>
+      </c>
+      <c r="AN54">
+        <v>1038.6948866828891</v>
+      </c>
+    </row>
+    <row r="55" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A55">
         <v>207</v>
       </c>
@@ -23398,8 +23440,14 @@
       <c r="AI55" s="4">
         <v>7.7965968009799376</v>
       </c>
-    </row>
-    <row r="56" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="AM55">
+        <v>12.618307944649743</v>
+      </c>
+      <c r="AN55">
+        <v>1038.6948866828891</v>
+      </c>
+    </row>
+    <row r="56" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A56">
         <v>208</v>
       </c>
@@ -23515,8 +23563,14 @@
       <c r="AI56" s="4">
         <v>8.0729738740265073</v>
       </c>
-    </row>
-    <row r="57" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="AM56">
+        <v>12.618307944649743</v>
+      </c>
+      <c r="AN56">
+        <v>1038.6948866828891</v>
+      </c>
+    </row>
+    <row r="57" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A57">
         <v>209</v>
       </c>
@@ -23632,8 +23686,14 @@
       <c r="AI57" s="4">
         <v>8.5932709261319697</v>
       </c>
-    </row>
-    <row r="58" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="AM57">
+        <v>12.618307944649743</v>
+      </c>
+      <c r="AN57">
+        <v>1038.6948866828891</v>
+      </c>
+    </row>
+    <row r="58" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A58">
         <v>210</v>
       </c>
@@ -23749,8 +23809,14 @@
       <c r="AI58" s="4">
         <v>10.514140761220755</v>
       </c>
-    </row>
-    <row r="59" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="AM58">
+        <v>12.618307944649743</v>
+      </c>
+      <c r="AN58">
+        <v>1038.6948866828891</v>
+      </c>
+    </row>
+    <row r="59" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A59">
         <v>211</v>
       </c>
@@ -23865,8 +23931,14 @@
       <c r="AI59" s="4">
         <v>8.3454167538624482</v>
       </c>
-    </row>
-    <row r="60" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="AM59">
+        <v>12.618307944649743</v>
+      </c>
+      <c r="AN59">
+        <v>1038.6948866828891</v>
+      </c>
+    </row>
+    <row r="60" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A60">
         <v>212</v>
       </c>
@@ -23981,8 +24053,14 @@
       <c r="AI60" s="4">
         <v>7.365802644416247</v>
       </c>
-    </row>
-    <row r="61" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="AM60">
+        <v>12.618307944649743</v>
+      </c>
+      <c r="AN60">
+        <v>1038.6948866828891</v>
+      </c>
+    </row>
+    <row r="61" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A61">
         <v>213</v>
       </c>
@@ -24097,8 +24175,14 @@
       <c r="AI61">
         <v>8.2818139636239732</v>
       </c>
-    </row>
-    <row r="62" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="AM61">
+        <v>12.618307944649743</v>
+      </c>
+      <c r="AN61">
+        <v>1038.6948866828891</v>
+      </c>
+    </row>
+    <row r="62" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A62">
         <v>214</v>
       </c>
@@ -24213,8 +24297,14 @@
       <c r="AI62">
         <v>7.7415180960311538</v>
       </c>
-    </row>
-    <row r="63" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="AM62">
+        <v>12.618307944649743</v>
+      </c>
+      <c r="AN62">
+        <v>1038.6948866828891</v>
+      </c>
+    </row>
+    <row r="63" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A63">
         <v>215</v>
       </c>
@@ -24329,8 +24419,14 @@
       <c r="AI63">
         <v>9.8787685577044435</v>
       </c>
-    </row>
-    <row r="64" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="AM63">
+        <v>12.618307944649743</v>
+      </c>
+      <c r="AN63">
+        <v>1038.6948866828891</v>
+      </c>
+    </row>
+    <row r="64" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A64">
         <v>216</v>
       </c>
@@ -24445,8 +24541,14 @@
       <c r="AI64">
         <v>8.9266938007326342</v>
       </c>
-    </row>
-    <row r="65" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="AM64">
+        <v>12.618307944649743</v>
+      </c>
+      <c r="AN64">
+        <v>1038.6948866828891</v>
+      </c>
+    </row>
+    <row r="65" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A65">
         <v>217</v>
       </c>
@@ -24561,8 +24663,14 @@
       <c r="AI65">
         <v>8.0562535528813406</v>
       </c>
-    </row>
-    <row r="66" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="AM65">
+        <v>12.618307944649743</v>
+      </c>
+      <c r="AN65">
+        <v>1038.6948866828891</v>
+      </c>
+    </row>
+    <row r="66" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A66">
         <v>218</v>
       </c>
@@ -24677,8 +24785,14 @@
       <c r="AI66">
         <v>7.7621726103869495</v>
       </c>
-    </row>
-    <row r="67" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="AM66">
+        <v>12.618307944649743</v>
+      </c>
+      <c r="AN66">
+        <v>1038.6948866828891</v>
+      </c>
+    </row>
+    <row r="67" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A67">
         <v>219</v>
       </c>
@@ -24790,8 +24904,14 @@
       <c r="AI67" s="4">
         <v>7.7366003545178721</v>
       </c>
-    </row>
-    <row r="68" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="AM67">
+        <v>12.618307944649743</v>
+      </c>
+      <c r="AN67">
+        <v>1038.6948866828891</v>
+      </c>
+    </row>
+    <row r="68" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A68">
         <v>220</v>
       </c>
@@ -24903,8 +25023,14 @@
       <c r="AI68" s="4">
         <v>9.6033750329605319</v>
       </c>
-    </row>
-    <row r="69" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="AM68">
+        <v>12.618307944649743</v>
+      </c>
+      <c r="AN68">
+        <v>1038.6948866828891</v>
+      </c>
+    </row>
+    <row r="69" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A69">
         <v>221</v>
       </c>
@@ -25001,8 +25127,14 @@
       <c r="AG69" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="70" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="AM69">
+        <v>12.618307944649743</v>
+      </c>
+      <c r="AN69">
+        <v>1038.6948866828891</v>
+      </c>
+    </row>
+    <row r="70" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A70">
         <v>222</v>
       </c>
@@ -25099,8 +25231,14 @@
       <c r="AG70" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="71" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="AM70">
+        <v>12.618307944649743</v>
+      </c>
+      <c r="AN70">
+        <v>1038.6948866828891</v>
+      </c>
+    </row>
+    <row r="71" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A71">
         <v>223</v>
       </c>
@@ -25197,8 +25335,14 @@
       <c r="AG71" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="72" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="AM71">
+        <v>12.618307944649743</v>
+      </c>
+      <c r="AN71">
+        <v>1038.6948866828891</v>
+      </c>
+    </row>
+    <row r="72" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A72">
         <v>224</v>
       </c>
@@ -25295,8 +25439,14 @@
       <c r="AG72" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="73" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="AM72">
+        <v>12.618307944649743</v>
+      </c>
+      <c r="AN72">
+        <v>1038.6948866828891</v>
+      </c>
+    </row>
+    <row r="73" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A73">
         <v>225</v>
       </c>
@@ -25396,8 +25546,14 @@
       <c r="AG73" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="74" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="AM73">
+        <v>12.618307944649743</v>
+      </c>
+      <c r="AN73">
+        <v>1038.6948866828891</v>
+      </c>
+    </row>
+    <row r="74" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A74">
         <v>226</v>
       </c>
@@ -25494,8 +25650,14 @@
       <c r="AG74" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="75" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="AM74">
+        <v>12.618307944649743</v>
+      </c>
+      <c r="AN74">
+        <v>1038.6948866828891</v>
+      </c>
+    </row>
+    <row r="75" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A75">
         <v>227</v>
       </c>
@@ -25592,8 +25754,14 @@
       <c r="AG75" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="76" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="AM75">
+        <v>12.618307944649743</v>
+      </c>
+      <c r="AN75">
+        <v>1038.6948866828891</v>
+      </c>
+    </row>
+    <row r="76" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A76">
         <v>228</v>
       </c>
@@ -25690,8 +25858,14 @@
       <c r="AG76" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="77" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="AM76">
+        <v>12.618307944649743</v>
+      </c>
+      <c r="AN76">
+        <v>1038.6948866828891</v>
+      </c>
+    </row>
+    <row r="77" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A77">
         <v>229</v>
       </c>
@@ -25789,8 +25963,14 @@
       <c r="AG77" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="78" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="AM77">
+        <v>12.618307944649743</v>
+      </c>
+      <c r="AN77">
+        <v>1038.6948866828891</v>
+      </c>
+    </row>
+    <row r="78" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A78">
         <v>230</v>
       </c>
@@ -25887,8 +26067,14 @@
       <c r="AG78" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="79" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="AM78">
+        <v>12.618307944649743</v>
+      </c>
+      <c r="AN78">
+        <v>1038.6948866828891</v>
+      </c>
+    </row>
+    <row r="79" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A79">
         <v>231</v>
       </c>
@@ -26000,8 +26186,14 @@
       <c r="AI79" s="4">
         <v>11.011816202365111</v>
       </c>
-    </row>
-    <row r="80" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="AM79">
+        <v>12.618307944649743</v>
+      </c>
+      <c r="AN79">
+        <v>1038.6948866828891</v>
+      </c>
+    </row>
+    <row r="80" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A80">
         <v>232</v>
       </c>
@@ -26098,8 +26290,14 @@
       <c r="AG80" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="81" spans="1:33" x14ac:dyDescent="0.35">
+      <c r="AM80">
+        <v>12.618307944649743</v>
+      </c>
+      <c r="AN80">
+        <v>1038.6948866828891</v>
+      </c>
+    </row>
+    <row r="81" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A81">
         <v>233</v>
       </c>
@@ -26194,8 +26392,14 @@
       <c r="AG81" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="82" spans="1:33" x14ac:dyDescent="0.35">
+      <c r="AM81">
+        <v>12.618307944649743</v>
+      </c>
+      <c r="AN81">
+        <v>1038.6948866828891</v>
+      </c>
+    </row>
+    <row r="82" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A82">
         <v>234</v>
       </c>
@@ -26292,8 +26496,14 @@
       <c r="AG82" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="83" spans="1:33" x14ac:dyDescent="0.35">
+      <c r="AM82">
+        <v>12.618307944649743</v>
+      </c>
+      <c r="AN82">
+        <v>1038.6948866828891</v>
+      </c>
+    </row>
+    <row r="83" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A83">
         <v>235</v>
       </c>
@@ -26390,8 +26600,14 @@
       <c r="AG83" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="84" spans="1:33" x14ac:dyDescent="0.35">
+      <c r="AM83">
+        <v>12.618307944649743</v>
+      </c>
+      <c r="AN83">
+        <v>1038.6948866828891</v>
+      </c>
+    </row>
+    <row r="84" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A84">
         <v>236</v>
       </c>
@@ -26488,8 +26704,14 @@
       <c r="AG84" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="85" spans="1:33" x14ac:dyDescent="0.35">
+      <c r="AM84">
+        <v>12.618307944649743</v>
+      </c>
+      <c r="AN84">
+        <v>1038.6948866828891</v>
+      </c>
+    </row>
+    <row r="85" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A85">
         <v>237</v>
       </c>
@@ -26586,8 +26808,14 @@
       <c r="AG85" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="86" spans="1:33" x14ac:dyDescent="0.35">
+      <c r="AM85">
+        <v>12.618307944649743</v>
+      </c>
+      <c r="AN85">
+        <v>1038.6948866828891</v>
+      </c>
+    </row>
+    <row r="86" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A86">
         <v>238</v>
       </c>
@@ -26684,8 +26912,14 @@
       <c r="AG86" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="87" spans="1:33" x14ac:dyDescent="0.35">
+      <c r="AM86">
+        <v>12.618307944649743</v>
+      </c>
+      <c r="AN86">
+        <v>1038.6948866828891</v>
+      </c>
+    </row>
+    <row r="87" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A87">
         <v>239</v>
       </c>
@@ -26782,8 +27016,14 @@
       <c r="AG87" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="88" spans="1:33" x14ac:dyDescent="0.35">
+      <c r="AM87">
+        <v>12.618307944649743</v>
+      </c>
+      <c r="AN87">
+        <v>1038.6948866828891</v>
+      </c>
+    </row>
+    <row r="88" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A88">
         <v>240</v>
       </c>
@@ -26880,8 +27120,14 @@
       <c r="AG88" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="89" spans="1:33" x14ac:dyDescent="0.35">
+      <c r="AM88">
+        <v>12.618307944649743</v>
+      </c>
+      <c r="AN88">
+        <v>1038.6948866828891</v>
+      </c>
+    </row>
+    <row r="89" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A89">
         <v>241</v>
       </c>
@@ -26978,8 +27224,14 @@
       <c r="AG89" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="90" spans="1:33" x14ac:dyDescent="0.35">
+      <c r="AM89">
+        <v>12.618307944649743</v>
+      </c>
+      <c r="AN89">
+        <v>1038.6948866828891</v>
+      </c>
+    </row>
+    <row r="90" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A90">
         <v>242</v>
       </c>
@@ -27076,8 +27328,14 @@
       <c r="AG90" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="91" spans="1:33" x14ac:dyDescent="0.35">
+      <c r="AM90">
+        <v>12.618307944649743</v>
+      </c>
+      <c r="AN90">
+        <v>1038.6948866828891</v>
+      </c>
+    </row>
+    <row r="91" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A91">
         <v>243</v>
       </c>
@@ -27174,8 +27432,14 @@
       <c r="AG91" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="92" spans="1:33" x14ac:dyDescent="0.35">
+      <c r="AM91">
+        <v>12.618307944649743</v>
+      </c>
+      <c r="AN91">
+        <v>1038.6948866828891</v>
+      </c>
+    </row>
+    <row r="92" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A92">
         <v>244</v>
       </c>
@@ -27272,8 +27536,14 @@
       <c r="AG92" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="93" spans="1:33" x14ac:dyDescent="0.35">
+      <c r="AM92">
+        <v>12.618307944649743</v>
+      </c>
+      <c r="AN92">
+        <v>1038.6948866828891</v>
+      </c>
+    </row>
+    <row r="93" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A93">
         <v>245</v>
       </c>
@@ -27365,8 +27635,14 @@
       <c r="AG93" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="94" spans="1:33" x14ac:dyDescent="0.35">
+      <c r="AM93">
+        <v>12.618307944649743</v>
+      </c>
+      <c r="AN93">
+        <v>1038.6948866828891</v>
+      </c>
+    </row>
+    <row r="94" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A94">
         <v>246</v>
       </c>
@@ -27462,8 +27738,14 @@
       <c r="AG94" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="95" spans="1:33" x14ac:dyDescent="0.35">
+      <c r="AM94">
+        <v>12.618307944649743</v>
+      </c>
+      <c r="AN94">
+        <v>1038.6948866828891</v>
+      </c>
+    </row>
+    <row r="95" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A95">
         <v>247</v>
       </c>
@@ -27561,8 +27843,14 @@
       <c r="AG95" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="96" spans="1:33" x14ac:dyDescent="0.35">
+      <c r="AM95">
+        <v>19.410673976313994</v>
+      </c>
+      <c r="AN95">
+        <v>497.82735437242388</v>
+      </c>
+    </row>
+    <row r="96" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A96">
         <v>248</v>
       </c>
@@ -27659,8 +27947,14 @@
       <c r="AG96" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="97" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="AM96">
+        <v>19.410673976313994</v>
+      </c>
+      <c r="AN96">
+        <v>497.82735437242388</v>
+      </c>
+    </row>
+    <row r="97" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A97">
         <v>249</v>
       </c>
@@ -27758,8 +28052,14 @@
       <c r="AG97" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="98" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="AM97">
+        <v>19.410673976313994</v>
+      </c>
+      <c r="AN97">
+        <v>497.82735437242388</v>
+      </c>
+    </row>
+    <row r="98" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A98">
         <v>250</v>
       </c>
@@ -27875,8 +28175,14 @@
       <c r="AI98">
         <v>8.3955777172979467</v>
       </c>
-    </row>
-    <row r="99" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="AM98">
+        <v>19.410673976313994</v>
+      </c>
+      <c r="AN98">
+        <v>497.82735437242388</v>
+      </c>
+    </row>
+    <row r="99" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A99">
         <v>251</v>
       </c>
@@ -27991,8 +28297,14 @@
       <c r="AI99">
         <v>8.1132993544354353</v>
       </c>
-    </row>
-    <row r="100" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="AM99">
+        <v>19.410673976313994</v>
+      </c>
+      <c r="AN99">
+        <v>497.82735437242388</v>
+      </c>
+    </row>
+    <row r="100" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A100">
         <v>252</v>
       </c>
@@ -28107,8 +28419,14 @@
       <c r="AI100">
         <v>9.3532259146514782</v>
       </c>
-    </row>
-    <row r="101" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="AM100">
+        <v>19.410673976313994</v>
+      </c>
+      <c r="AN100">
+        <v>497.82735437242388</v>
+      </c>
+    </row>
+    <row r="101" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A101">
         <v>253</v>
       </c>
@@ -28223,8 +28541,14 @@
       <c r="AI101">
         <v>8.6385141480541829</v>
       </c>
-    </row>
-    <row r="102" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="AM101">
+        <v>19.410673976313994</v>
+      </c>
+      <c r="AN101">
+        <v>497.82735437242388</v>
+      </c>
+    </row>
+    <row r="102" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A102">
         <v>254</v>
       </c>
@@ -28339,8 +28663,14 @@
       <c r="AI102">
         <v>8.1024803231062119</v>
       </c>
-    </row>
-    <row r="103" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="AM102">
+        <v>19.410673976313994</v>
+      </c>
+      <c r="AN102">
+        <v>497.82735437242388</v>
+      </c>
+    </row>
+    <row r="103" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A103">
         <v>255</v>
       </c>
@@ -28455,8 +28785,14 @@
       <c r="AI103">
         <v>7.988388719998019</v>
       </c>
-    </row>
-    <row r="104" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="AM103">
+        <v>19.410673976313994</v>
+      </c>
+      <c r="AN103">
+        <v>497.82735437242388</v>
+      </c>
+    </row>
+    <row r="104" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A104">
         <v>256</v>
       </c>
@@ -28572,8 +28908,14 @@
       <c r="AI104">
         <v>7.9028200176668761</v>
       </c>
-    </row>
-    <row r="105" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="AM104">
+        <v>19.410673976313994</v>
+      </c>
+      <c r="AN104">
+        <v>497.82735437242388</v>
+      </c>
+    </row>
+    <row r="105" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A105">
         <v>257</v>
       </c>
@@ -28688,8 +29030,14 @@
       <c r="AI105">
         <v>8.7122802707534444</v>
       </c>
-    </row>
-    <row r="106" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="AM105">
+        <v>19.410673976313994</v>
+      </c>
+      <c r="AN105">
+        <v>497.82735437242388</v>
+      </c>
+    </row>
+    <row r="106" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A106">
         <v>258</v>
       </c>
@@ -28804,8 +29152,14 @@
       <c r="AI106">
         <v>8.1349374170938873</v>
       </c>
-    </row>
-    <row r="107" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="AM106">
+        <v>19.410673976313994</v>
+      </c>
+      <c r="AN106">
+        <v>497.82735437242388</v>
+      </c>
+    </row>
+    <row r="107" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A107">
         <v>259</v>
       </c>
@@ -28905,8 +29259,14 @@
       <c r="AG107" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="108" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="AM107">
+        <v>19.410673976313994</v>
+      </c>
+      <c r="AN107">
+        <v>497.82735437242388</v>
+      </c>
+    </row>
+    <row r="108" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A108">
         <v>260</v>
       </c>
@@ -29021,8 +29381,14 @@
       <c r="AI108">
         <v>8.1447729001204543</v>
       </c>
-    </row>
-    <row r="109" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="AM108">
+        <v>19.410673976313994</v>
+      </c>
+      <c r="AN108">
+        <v>497.82735437242388</v>
+      </c>
+    </row>
+    <row r="109" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A109">
         <v>261</v>
       </c>
@@ -29137,8 +29503,14 @@
       <c r="AI109">
         <v>8.5726164117761758</v>
       </c>
-    </row>
-    <row r="110" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="AM109">
+        <v>19.410673976313994</v>
+      </c>
+      <c r="AN109">
+        <v>497.82735437242388</v>
+      </c>
+    </row>
+    <row r="110" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A110">
         <v>262</v>
       </c>
@@ -29253,8 +29625,14 @@
       <c r="AI110">
         <v>9.6348485786455509</v>
       </c>
-    </row>
-    <row r="111" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="AM110">
+        <v>19.410673976313994</v>
+      </c>
+      <c r="AN110">
+        <v>497.82735437242388</v>
+      </c>
+    </row>
+    <row r="111" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A111">
         <v>263</v>
       </c>
@@ -29369,8 +29747,14 @@
       <c r="AI111">
         <v>8.1634603178709337</v>
       </c>
-    </row>
-    <row r="112" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="AM111">
+        <v>19.410673976313994</v>
+      </c>
+      <c r="AN111">
+        <v>497.82735437242388</v>
+      </c>
+    </row>
+    <row r="112" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A112">
         <v>264</v>
       </c>
@@ -29485,8 +29869,14 @@
       <c r="AI112">
         <v>8.3945941689952903</v>
       </c>
-    </row>
-    <row r="113" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="AM112">
+        <v>19.410673976313994</v>
+      </c>
+      <c r="AN112">
+        <v>497.82735437242388</v>
+      </c>
+    </row>
+    <row r="113" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A113">
         <v>265</v>
       </c>
@@ -29601,8 +29991,14 @@
       <c r="AI113">
         <v>9.8177885629397217</v>
       </c>
-    </row>
-    <row r="114" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="AM113">
+        <v>19.410673976313994</v>
+      </c>
+      <c r="AN113">
+        <v>497.82735437242388</v>
+      </c>
+    </row>
+    <row r="114" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A114">
         <v>266</v>
       </c>
@@ -29697,8 +30093,14 @@
       <c r="AG114" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="115" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="AM114">
+        <v>19.410673976313994</v>
+      </c>
+      <c r="AN114">
+        <v>497.82735437242388</v>
+      </c>
+    </row>
+    <row r="115" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A115">
         <v>267</v>
       </c>
@@ -29794,8 +30196,14 @@
       <c r="AG115" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="116" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="AM115">
+        <v>19.410673976313994</v>
+      </c>
+      <c r="AN115">
+        <v>497.82735437242388</v>
+      </c>
+    </row>
+    <row r="116" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A116">
         <v>268</v>
       </c>
@@ -29893,8 +30301,14 @@
       <c r="AG116" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="117" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="AM116">
+        <v>19.410673976313994</v>
+      </c>
+      <c r="AN116">
+        <v>497.82735437242388</v>
+      </c>
+    </row>
+    <row r="117" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A117">
         <v>269</v>
       </c>
@@ -29991,8 +30405,14 @@
       <c r="AG117" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="118" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="AM117">
+        <v>19.410673976313994</v>
+      </c>
+      <c r="AN117">
+        <v>497.82735437242388</v>
+      </c>
+    </row>
+    <row r="118" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A118">
         <v>270</v>
       </c>
@@ -30104,8 +30524,14 @@
       <c r="AI118">
         <v>9.4627276256806052</v>
       </c>
-    </row>
-    <row r="119" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="AM118">
+        <v>19.410673976313994</v>
+      </c>
+      <c r="AN118">
+        <v>497.82735437242388</v>
+      </c>
+    </row>
+    <row r="119" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A119">
         <v>271</v>
       </c>
@@ -30218,7 +30644,7 @@
         <v>11.333436497333894</v>
       </c>
     </row>
-    <row r="120" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A120">
         <v>272</v>
       </c>
@@ -30332,7 +30758,7 @@
         <v>10.690195907396328</v>
       </c>
     </row>
-    <row r="121" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A121">
         <v>273</v>
       </c>
@@ -30446,7 +30872,7 @@
         <v>11.608830022077806</v>
       </c>
     </row>
-    <row r="122" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A122">
         <v>274</v>
       </c>
@@ -30560,7 +30986,7 @@
         <v>11.457363583468654</v>
       </c>
     </row>
-    <row r="123" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A123">
         <v>275</v>
       </c>
@@ -30674,7 +31100,7 @@
         <v>9.2148734534110854</v>
       </c>
     </row>
-    <row r="124" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A124">
         <v>276</v>
       </c>
@@ -30788,7 +31214,7 @@
         <v>13.488390828455005</v>
       </c>
     </row>
-    <row r="125" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A125">
         <v>277</v>
       </c>
@@ -30902,7 +31328,7 @@
         <v>11.191805541751311</v>
       </c>
     </row>
-    <row r="126" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A126">
         <v>278</v>
       </c>
@@ -31015,7 +31441,7 @@
         <v>7.493663923761634</v>
       </c>
     </row>
-    <row r="127" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A127">
         <v>279</v>
       </c>
@@ -31128,7 +31554,7 @@
         <v>5.0072538146451713</v>
       </c>
     </row>
-    <row r="128" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A128">
         <v>280</v>
       </c>

</xml_diff>